<commit_message>
Actualización automática 2026-09-14 12:30:18
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2160,7 +2160,7 @@
         <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>1740.39</v>
+        <v>1728.65</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -3954,7 +3954,7 @@
         <v>0</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>0</v>
+        <v>-37.22</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>253.96</v>
@@ -5233,7 +5233,7 @@
         <v>0</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>1740.39</v>
+        <v>1728.65</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>3000</v>
@@ -5854,7 +5854,7 @@
         <v>2665.26</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>2737.54</v>
+        <v>2700.32</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>3000</v>
@@ -6060,7 +6060,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>26475.88</v>
+        <v>26426.92</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6351,13 +6351,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1210.83</v>
+        <v>1173.61</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-482.8299999999999</v>
+        <v>-445.6099999999999</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>1.663228021978022</v>
+        <v>1.612101648351648</v>
       </c>
     </row>
     <row r="12">
@@ -6423,13 +6423,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>11214.06</v>
+        <v>11202.32</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>46907.94</v>
+        <v>46919.68</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.1929400227108496</v>
+        <v>0.1927380337909914</v>
       </c>
     </row>
     <row r="15">
@@ -6466,13 +6466,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>26475.88</v>
+        <v>26426.92</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>54913.12</v>
+        <v>54962.08</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3253004705795623</v>
+        <v>0.3246989150868053</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-14 14:30:20
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -1140,7 +1140,7 @@
         <v>0</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>74.61</v>
+        <v>174.09</v>
       </c>
       <c r="N11" s="2" t="n">
         <v>0</v>
@@ -1500,7 +1500,7 @@
         <v>0</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>70.2</v>
+        <v>1030.33</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
@@ -3774,7 +3774,7 @@
         <v>0</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>874.62</v>
+        <v>2210.72</v>
       </c>
       <c r="L55" s="2" t="n">
         <v>0</v>
@@ -4936,7 +4936,7 @@
         <v>4036.83</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>74.61</v>
+        <v>174.09</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>5000</v>
@@ -5071,7 +5071,7 @@
         <v>1205.88</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>70.2</v>
+        <v>1030.33</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>1500</v>
@@ -5773,7 +5773,7 @@
         <v>0</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>944.55</v>
+        <v>2280.65</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>1500</v>
@@ -6060,7 +6060,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>26426.92</v>
+        <v>28822.63</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6351,13 +6351,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1173.61</v>
+        <v>2509.71</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-445.6099999999999</v>
+        <v>-1781.71</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>1.612101648351648</v>
+        <v>3.447403846153846</v>
       </c>
     </row>
     <row r="12">
@@ -6423,13 +6423,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>11202.32</v>
+        <v>12261.93</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>46919.68</v>
+        <v>45860.07</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.1927380337909914</v>
+        <v>0.2109688241973779</v>
       </c>
     </row>
     <row r="15">
@@ -6466,13 +6466,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>26426.92</v>
+        <v>28822.63</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>54962.08</v>
+        <v>52566.37</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3246989150868053</v>
+        <v>0.3541342196119869</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-15 15:30:18
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -3948,7 +3948,7 @@
         <v>0</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>1588.78</v>
+        <v>1499.57</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0</v>
@@ -5854,7 +5854,7 @@
         <v>2665.26</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>2817.41</v>
+        <v>2728.2</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>3000</v>
@@ -6060,7 +6060,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>28939.72</v>
+        <v>28850.51</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6279,13 +6279,13 @@
         <v>1676</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>3875.86</v>
+        <v>3786.65</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-2199.86</v>
+        <v>-2110.65</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>2.312565632458234</v>
+        <v>2.259337708830549</v>
       </c>
     </row>
     <row r="9">
@@ -6466,13 +6466,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>28939.72</v>
+        <v>28850.51</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>52449.28</v>
+        <v>52538.49</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3555728661121282</v>
+        <v>0.3544767720453624</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-16 08:30:18
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R70"/>
+  <dimension ref="A1:R69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1260,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0</v>
+        <v>1112.55</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>LAND EXPEDITIONS TIPS TRANSPORTE TURISTICOS S.A.</t>
+          <t>MAD&amp;DECO S.A.</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="L41" s="2" t="n">
-        <v>0</v>
+        <v>909.35</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>0</v>
+        <v>4300.47</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -2966,7 +2966,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>MAD&amp;DECO S.A.</t>
+          <t>MAJACSA S.A.</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -2997,10 +2997,10 @@
         <v>0</v>
       </c>
       <c r="L42" s="2" t="n">
-        <v>909.35</v>
+        <v>0</v>
       </c>
       <c r="M42" s="2" t="n">
-        <v>4300.47</v>
+        <v>0</v>
       </c>
       <c r="N42" s="2" t="n">
         <v>0</v>
@@ -3026,7 +3026,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>MAJACSA S.A.</t>
+          <t>MEGAMETALES S.A.</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3060,7 +3060,7 @@
         <v>0</v>
       </c>
       <c r="M43" s="2" t="n">
-        <v>0</v>
+        <v>1324.05</v>
       </c>
       <c r="N43" s="2" t="n">
         <v>0</v>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>MEGAMETALES S.A.</t>
+          <t>MONCAYO PINCAY JOSE GREGORIO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3120,7 +3120,7 @@
         <v>0</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>1324.05</v>
+        <v>0</v>
       </c>
       <c r="N44" s="2" t="n">
         <v>0</v>
@@ -3146,7 +3146,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MONCAYO PINCAY JOSE GREGORIO</t>
+          <t>MUNDO &amp; PIEDRA S.A. MUNPIEDSA</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MUNDO &amp; PIEDRA S.A. MUNPIEDSA</t>
+          <t>PEREZ NARANJO JOYCE LORENA</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3234,7 +3234,7 @@
         <v>0</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>0</v>
+        <v>379.64</v>
       </c>
       <c r="L46" s="2" t="n">
         <v>0</v>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PEREZ NARANJO JOYCE LORENA</t>
+          <t>PERUCCI .S.A</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3294,7 +3294,7 @@
         <v>0</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>379.64</v>
+        <v>0</v>
       </c>
       <c r="L47" s="2" t="n">
         <v>0</v>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PERUCCI .S.A</t>
+          <t>PIEDRA VALDEZ GENESIS DAYANNA</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3386,7 +3386,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PIEDRA VALDEZ GENESIS DAYANNA</t>
+          <t>PORCEKER S.A.</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3446,7 +3446,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PORCEKER S.A.</t>
+          <t>QUIROZ PEÑAFIEL DIANA ISABEL</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>QUIROZ PEÑAFIEL DIANA ISABEL</t>
+          <t>RAMOS BARRENO LIZ TAMARA</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>RAMOS BARRENO LIZ TAMARA</t>
+          <t>RAMOS RODRIGUEZ ADRIANA CAROLINA</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3600,7 +3600,7 @@
         <v>0</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>0</v>
+        <v>-454.9</v>
       </c>
       <c r="N52" s="2" t="n">
         <v>0</v>
@@ -3626,7 +3626,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>RAMOS RODRIGUEZ ADRIANA CAROLINA</t>
+          <t>RIOFRIO SALCEDO JUAN ANTONIO</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3660,7 +3660,7 @@
         <v>0</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>-454.9</v>
+        <v>0</v>
       </c>
       <c r="N53" s="2" t="n">
         <v>0</v>
@@ -3686,7 +3686,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>RIOFRIO SALCEDO JUAN ANTONIO</t>
+          <t>RIVERA CANTOS MARTHA JACQUELIN</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3714,13 +3714,13 @@
         <v>0</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>0</v>
+        <v>2210.72</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>0</v>
+        <v>69.93000000000001</v>
       </c>
       <c r="N54" s="2" t="n">
         <v>0</v>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>RIVERA CANTOS MARTHA JACQUELIN</t>
+          <t>RUIZ PINEDA LUIS ALFREDO</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3774,13 +3774,13 @@
         <v>0</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>2210.72</v>
+        <v>0</v>
       </c>
       <c r="L55" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>69.93000000000001</v>
+        <v>0</v>
       </c>
       <c r="N55" s="2" t="n">
         <v>0</v>
@@ -3806,7 +3806,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>RUIZ PINEDA LUIS ALFREDO</t>
+          <t>SALAZAR BALLADARES MARIA ANGELICA</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3825,10 +3825,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>0</v>
+        <v>208.8</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>0</v>
+        <v>479.12</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0</v>
@@ -3837,10 +3837,10 @@
         <v>0</v>
       </c>
       <c r="L56" s="2" t="n">
-        <v>0</v>
+        <v>423.26</v>
       </c>
       <c r="M56" s="2" t="n">
-        <v>0</v>
+        <v>359.32</v>
       </c>
       <c r="N56" s="2" t="n">
         <v>0</v>
@@ -3866,7 +3866,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>SALAZAR BALLADARES MARIA ANGELICA</t>
+          <t>SANCHEZ CORREA MARCO EDUARDO</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3885,22 +3885,22 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>208.8</v>
+        <v>0</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>479.12</v>
+        <v>1499.57</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>0</v>
+        <v>-37.22</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>423.26</v>
+        <v>253.96</v>
       </c>
       <c r="M57" s="2" t="n">
-        <v>359.32</v>
+        <v>1011.89</v>
       </c>
       <c r="N57" s="2" t="n">
         <v>0</v>
@@ -3926,7 +3926,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>SANCHEZ CORREA MARCO EDUARDO</t>
+          <t>SANTISTEVAN CABRERA BLADIMIR ADOLFO</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3948,19 +3948,19 @@
         <v>0</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>1499.57</v>
+        <v>0</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>-37.22</v>
+        <v>0</v>
       </c>
       <c r="L58" s="2" t="n">
-        <v>253.96</v>
+        <v>0</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>1011.89</v>
+        <v>0</v>
       </c>
       <c r="N58" s="2" t="n">
         <v>0</v>
@@ -3986,7 +3986,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>SANTISTEVAN CABRERA BLADIMIR ADOLFO</t>
+          <t>SERVICERAMICAS S.A.S.</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4017,7 +4017,7 @@
         <v>0</v>
       </c>
       <c r="L59" s="2" t="n">
-        <v>0</v>
+        <v>1219.77</v>
       </c>
       <c r="M59" s="2" t="n">
         <v>0</v>
@@ -4046,7 +4046,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>SERVICERAMICAS S.A.S.</t>
+          <t>SILVA MERA DAVID ALEXANDER</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -4077,7 +4077,7 @@
         <v>0</v>
       </c>
       <c r="L60" s="2" t="n">
-        <v>1219.77</v>
+        <v>0</v>
       </c>
       <c r="M60" s="2" t="n">
         <v>0</v>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>SILVA MERA DAVID ALEXANDER</t>
+          <t>SISA GUANO CARLOS ALBERTO</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>SISA GUANO CARLOS ALBERTO</t>
+          <t>SUSANDECORATIONS S.A.S.</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -4226,7 +4226,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>SUSANDECORATIONS S.A.S.</t>
+          <t>TAPIA BALLADARES LORENA ELIZABETH</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -4260,7 +4260,7 @@
         <v>0</v>
       </c>
       <c r="M63" s="2" t="n">
-        <v>0</v>
+        <v>1562.9</v>
       </c>
       <c r="N63" s="2" t="n">
         <v>0</v>
@@ -4286,7 +4286,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>TAPIA BALLADARES LORENA ELIZABETH</t>
+          <t>TAPIA TAPIA ANGEL GUSTAVO</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -4320,7 +4320,7 @@
         <v>0</v>
       </c>
       <c r="M64" s="2" t="n">
-        <v>1562.9</v>
+        <v>0</v>
       </c>
       <c r="N64" s="2" t="n">
         <v>0</v>
@@ -4346,7 +4346,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>TAPIA TAPIA ANGEL GUSTAVO</t>
+          <t>TRANSCASH S.A.</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -4406,7 +4406,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>TRANSCASH S.A.</t>
+          <t>VERDUGA PINCAY ANGEL ADRIAN</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -4466,7 +4466,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>VERDUGA PINCAY ANGEL ADRIAN</t>
+          <t>VILLACIS RAMIREZ PAOLA</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -4526,7 +4526,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>VILLACIS RAMIREZ PAOLA</t>
+          <t>VIZUETA CAZORLA SUSANA JOHANNA</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -4545,10 +4545,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>0</v>
+        <v>221.4</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>0</v>
+        <v>223.02</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0</v>
@@ -4579,144 +4579,84 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>CASTRO ALCIVAR EDA MARIA</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>VIZUETA CAZORLA SUSANA JOHANNA</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H69" s="2" t="n">
-        <v>221.4</v>
-      </c>
-      <c r="I69" s="2" t="n">
-        <v>223.02</v>
-      </c>
-      <c r="J69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R69" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="C70" s="4" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="D70" s="4" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="E70" s="4" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="F70" s="4" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="G70" s="4" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="H70" s="4" t="inlineStr">
-        <is>
-          <t>5 de 68</t>
-        </is>
-      </c>
-      <c r="I70" s="4" t="inlineStr">
-        <is>
-          <t>5 de 68</t>
-        </is>
-      </c>
-      <c r="J70" s="4" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="K70" s="4" t="inlineStr">
-        <is>
-          <t>2 de 68</t>
-        </is>
-      </c>
-      <c r="L70" s="4" t="inlineStr">
-        <is>
-          <t>4 de 68</t>
-        </is>
-      </c>
-      <c r="M70" s="4" t="inlineStr">
-        <is>
-          <t>11 de 68</t>
-        </is>
-      </c>
-      <c r="N70" s="4" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="O70" s="4" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="P70" s="4" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="Q70" s="4" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
-        </is>
-      </c>
-      <c r="R70" s="4" t="inlineStr">
-        <is>
-          <t>0 de 68</t>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>0 de 67</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>0 de 67</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>0 de 67</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>0 de 67</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>0 de 67</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>5 de 67</t>
+        </is>
+      </c>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>5 de 67</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr">
+        <is>
+          <t>0 de 67</t>
+        </is>
+      </c>
+      <c r="K69" s="4" t="inlineStr">
+        <is>
+          <t>2 de 67</t>
+        </is>
+      </c>
+      <c r="L69" s="4" t="inlineStr">
+        <is>
+          <t>4 de 67</t>
+        </is>
+      </c>
+      <c r="M69" s="4" t="inlineStr">
+        <is>
+          <t>12 de 67</t>
+        </is>
+      </c>
+      <c r="N69" s="4" t="inlineStr">
+        <is>
+          <t>0 de 67</t>
+        </is>
+      </c>
+      <c r="O69" s="4" t="inlineStr">
+        <is>
+          <t>0 de 67</t>
+        </is>
+      </c>
+      <c r="P69" s="4" t="inlineStr">
+        <is>
+          <t>0 de 67</t>
+        </is>
+      </c>
+      <c r="Q69" s="4" t="inlineStr">
+        <is>
+          <t>0 de 67</t>
+        </is>
+      </c>
+      <c r="R69" s="4" t="inlineStr">
+        <is>
+          <t>0 de 67</t>
         </is>
       </c>
     </row>
@@ -4990,7 +4930,7 @@
         <v>0</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>1122.88</v>
+        <v>2235.43</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>0</v>
@@ -6060,7 +6000,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>28850.51</v>
+        <v>29963.06</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6423,13 +6363,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>12261.93</v>
+        <v>13374.48</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>45860.07</v>
+        <v>44747.52</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.2109688241973779</v>
+        <v>0.2301104573139259</v>
       </c>
     </row>
     <row r="15">
@@ -6466,13 +6406,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>28850.51</v>
+        <v>29963.06</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>52538.49</v>
+        <v>51425.94</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3544767720453624</v>
+        <v>0.3681463096978707</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-16 12:30:18
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -1260,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>1112.55</v>
+        <v>2225.1</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -1620,7 +1620,7 @@
         <v>0</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>881.3099999999999</v>
+        <v>933.8099999999999</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -2940,7 +2940,7 @@
         <v>909.35</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>4300.47</v>
+        <v>6612.26</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -4930,7 +4930,7 @@
         <v>0</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>2235.43</v>
+        <v>3347.98</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>0</v>
@@ -5065,7 +5065,7 @@
         <v>4090.91</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>881.3099999999999</v>
+        <v>933.8099999999999</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>2000</v>
@@ -5443,7 +5443,7 @@
         <v>6566.73</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>5209.82</v>
+        <v>7521.61</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>6000</v>
@@ -6000,7 +6000,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>29963.06</v>
+        <v>33439.9</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6363,13 +6363,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>13374.48</v>
+        <v>16851.32</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>44747.52</v>
+        <v>41270.68</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.2301104573139259</v>
+        <v>0.2899301469323148</v>
       </c>
     </row>
     <row r="15">
@@ -6406,13 +6406,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>29963.06</v>
+        <v>33439.9</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>51425.94</v>
+        <v>47949.1</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3681463096978707</v>
+        <v>0.4108651046210176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-17 09:30:19
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -1260,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>2225.1</v>
+        <v>3337.65</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -4020,7 +4020,7 @@
         <v>1219.77</v>
       </c>
       <c r="M59" s="2" t="n">
-        <v>0</v>
+        <v>18.96</v>
       </c>
       <c r="N59" s="2" t="n">
         <v>0</v>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="M69" s="4" t="inlineStr">
         <is>
-          <t>12 de 67</t>
+          <t>13 de 67</t>
         </is>
       </c>
       <c r="N69" s="4" t="inlineStr">
@@ -4930,7 +4930,7 @@
         <v>0</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>3347.98</v>
+        <v>4460.53</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>0</v>
@@ -5821,7 +5821,7 @@
         <v>1696.95</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>1219.77</v>
+        <v>1238.73</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>2000</v>
@@ -6000,7 +6000,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>35195.89</v>
+        <v>36327.4</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6363,13 +6363,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>18536.21</v>
+        <v>19667.72</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>39585.79</v>
+        <v>38454.28</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.3189189979697877</v>
+        <v>0.3383868414713878</v>
       </c>
     </row>
     <row r="15">
@@ -6406,13 +6406,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>35195.89</v>
+        <v>36327.4</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>46193.11</v>
+        <v>45061.6</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.4324403789209844</v>
+        <v>0.4463428718868643</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-18 09:30:20
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2940,7 +2940,7 @@
         <v>909.35</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>7275.4</v>
+        <v>7296.12</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -5443,7 +5443,7 @@
         <v>6566.73</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>8184.75</v>
+        <v>8205.469999999999</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>6000</v>
@@ -6000,7 +6000,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>38033.61</v>
+        <v>38054.33</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6363,13 +6363,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>20330.86</v>
+        <v>20351.58</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>37791.14</v>
+        <v>37770.42</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.3497962905612333</v>
+        <v>0.3501527820790751</v>
       </c>
     </row>
     <row r="15">
@@ -6406,13 +6406,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>38033.61</v>
+        <v>38054.33</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>43355.39</v>
+        <v>43334.67</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.4673065156225043</v>
+        <v>0.4675610954797332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-18 10:30:18
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -1740,7 +1740,7 @@
         <v>0</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>273.89</v>
+        <v>2243.53</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
@@ -5092,7 +5092,7 @@
         <v>0</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>273.89</v>
+        <v>2243.53</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>2000</v>
@@ -6000,7 +6000,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>38054.33</v>
+        <v>40023.97</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6363,13 +6363,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>20351.58</v>
+        <v>22321.22</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>37770.42</v>
+        <v>35800.78</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.3501527820790751</v>
+        <v>0.3840408107085097</v>
       </c>
     </row>
     <row r="15">
@@ -6406,13 +6406,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>38054.33</v>
+        <v>40023.97</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>43334.67</v>
+        <v>41365.03</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.4675610954797332</v>
+        <v>0.4917614173905565</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-18 12:30:18
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -4233,7 +4233,7 @@
         <v>0</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>0</v>
@@ -4586,7 +4586,7 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>0 de 67</t>
+          <t>1 de 67</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
@@ -5902,7 +5902,7 @@
         <v>0</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>1562.9</v>
+        <v>1627.9</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>2000</v>
@@ -6000,7 +6000,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>40023.97</v>
+        <v>40088.97</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6099,13 +6099,13 @@
         <v>7842</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>7842</v>
+        <v>7777</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0</v>
+        <v>0.008288701861769956</v>
       </c>
     </row>
     <row r="4">
@@ -6406,13 +6406,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>40023.97</v>
+        <v>40088.97</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>41365.03</v>
+        <v>41300.03</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.4917614173905565</v>
+        <v>0.4925600511125582</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-18 14:30:18
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -777,7 +777,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>254.94</v>
+        <v>509.88</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>0</v>
@@ -4768,7 +4768,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>254.94</v>
+        <v>509.88</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>0</v>
@@ -6000,7 +6000,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>40088.97</v>
+        <v>40343.91</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6339,13 +6339,13 @@
         <v>2534</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>3841.39</v>
+        <v>4096.33</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-1307.39</v>
+        <v>-1562.33</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>1.515939226519337</v>
+        <v>1.616546961325967</v>
       </c>
     </row>
     <row r="14">
@@ -6406,13 +6406,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>40088.97</v>
+        <v>40343.91</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>41300.03</v>
+        <v>41045.09</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.4925600511125582</v>
+        <v>0.4956924154369756</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-18 15:30:19
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -1260,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3337.65</v>
+        <v>3297.92</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -1500,7 +1500,7 @@
         <v>0</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>1030.33</v>
+        <v>1872.91</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
@@ -2937,7 +2937,7 @@
         <v>0</v>
       </c>
       <c r="L41" s="2" t="n">
-        <v>909.35</v>
+        <v>1480.89</v>
       </c>
       <c r="M41" s="2" t="n">
         <v>7296.12</v>
@@ -3714,7 +3714,7 @@
         <v>0</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>2210.72</v>
+        <v>2124.4</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
@@ -3840,7 +3840,7 @@
         <v>423.26</v>
       </c>
       <c r="M56" s="2" t="n">
-        <v>2044.21</v>
+        <v>2026.04</v>
       </c>
       <c r="N56" s="2" t="n">
         <v>0</v>
@@ -4554,7 +4554,7 @@
         <v>0</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>0</v>
+        <v>446.69</v>
       </c>
       <c r="L68" s="2" t="n">
         <v>0</v>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="K69" s="4" t="inlineStr">
         <is>
-          <t>2 de 67</t>
+          <t>3 de 67</t>
         </is>
       </c>
       <c r="L69" s="4" t="inlineStr">
@@ -4930,7 +4930,7 @@
         <v>0</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>4460.53</v>
+        <v>4420.8</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>0</v>
@@ -5011,7 +5011,7 @@
         <v>1205.88</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>1030.33</v>
+        <v>1872.91</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>1500</v>
@@ -5443,7 +5443,7 @@
         <v>6566.73</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>8205.469999999999</v>
+        <v>8777.01</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>6000</v>
@@ -5713,7 +5713,7 @@
         <v>0</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>2280.65</v>
+        <v>2194.33</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>1500</v>
@@ -5767,7 +5767,7 @@
         <v>24.06</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>3226.49</v>
+        <v>3208.32</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>4000</v>
@@ -5983,7 +5983,7 @@
         <v>0</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>444.42</v>
+        <v>891.11</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>1000</v>
@@ -6000,7 +6000,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>40343.91</v>
+        <v>42060.5</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6023,7 +6023,7 @@
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
@@ -6291,13 +6291,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>2509.71</v>
+        <v>2870.08</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-1781.71</v>
+        <v>-2142.08</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>3.447403846153846</v>
+        <v>3.942417582417582</v>
       </c>
     </row>
     <row r="12">
@@ -6339,13 +6339,13 @@
         <v>2534</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>4096.33</v>
+        <v>4667.87</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-1562.33</v>
+        <v>-2133.87</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>1.616546961325967</v>
+        <v>1.842095501183899</v>
       </c>
     </row>
     <row r="14">
@@ -6363,13 +6363,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>22321.22</v>
+        <v>23105.9</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>35800.78</v>
+        <v>35016.1</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.3840408107085097</v>
+        <v>0.3975413784797495</v>
       </c>
     </row>
     <row r="15">
@@ -6406,13 +6406,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>40343.91</v>
+        <v>42060.5</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>41045.09</v>
+        <v>39328.5</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.4956924154369756</v>
+        <v>0.5167835948346828</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-21 10:30:18
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -3360,7 +3360,7 @@
         <v>0</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>0</v>
+        <v>59.62</v>
       </c>
       <c r="N48" s="2" t="n">
         <v>0</v>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="M69" s="4" t="inlineStr">
         <is>
-          <t>13 de 67</t>
+          <t>14 de 67</t>
         </is>
       </c>
       <c r="N69" s="4" t="inlineStr">
@@ -5605,7 +5605,7 @@
         <v>0</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0</v>
+        <v>59.62</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>0</v>
@@ -6000,7 +6000,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>42060.5</v>
+        <v>42120.12</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6023,7 +6023,7 @@
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
@@ -6363,13 +6363,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>23105.9</v>
+        <v>23165.52</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>35016.1</v>
+        <v>34956.48</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.3975413784797495</v>
+        <v>0.3985671518529988</v>
       </c>
     </row>
     <row r="15">
@@ -6406,13 +6406,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>42060.5</v>
+        <v>42120.12</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>39328.5</v>
+        <v>39268.88</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.5167835948346828</v>
+        <v>0.517516126257848</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-21 12:30:18
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -1569,7 +1569,7 @@
         <v>0</v>
       </c>
       <c r="P18" s="2" t="n">
-        <v>0</v>
+        <v>9.06</v>
       </c>
       <c r="Q18" s="2" t="n">
         <v>0</v>
@@ -4646,7 +4646,7 @@
       </c>
       <c r="P69" s="4" t="inlineStr">
         <is>
-          <t>0 de 67</t>
+          <t>1 de 67</t>
         </is>
       </c>
       <c r="Q69" s="4" t="inlineStr">
@@ -5038,7 +5038,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0</v>
+        <v>9.06</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>0</v>
@@ -6000,7 +6000,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>42120.12</v>
+        <v>42129.18</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6243,13 +6243,13 @@
         <v>250</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0</v>
+        <v>9.06</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>250</v>
+        <v>240.94</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0</v>
+        <v>0.03624</v>
       </c>
     </row>
     <row r="10">
@@ -6406,13 +6406,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>42120.12</v>
+        <v>42129.18</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>39268.88</v>
+        <v>39259.82000000001</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.517516126257848</v>
+        <v>0.5176274435120225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-23 16:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2757,7 +2757,7 @@
         <v>0</v>
       </c>
       <c r="L38" s="2" t="n">
-        <v>0</v>
+        <v>654.64</v>
       </c>
       <c r="M38" s="2" t="n">
         <v>0</v>
@@ -4626,7 +4626,7 @@
       </c>
       <c r="L69" s="4" t="inlineStr">
         <is>
-          <t>7 de 67</t>
+          <t>8 de 67</t>
         </is>
       </c>
       <c r="M69" s="4" t="inlineStr">
@@ -5362,7 +5362,7 @@
         <v>7198.47</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>2508.2</v>
+        <v>3162.84</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>0</v>
@@ -6000,7 +6000,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>48102.24</v>
+        <v>48756.88</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6339,13 +6339,13 @@
         <v>2534</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5895.32</v>
+        <v>6549.96</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-3361.32</v>
+        <v>-4015.96</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>2.326487766377269</v>
+        <v>2.584830307813733</v>
       </c>
     </row>
     <row r="14">
@@ -6406,13 +6406,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>48102.24</v>
+        <v>48756.88</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>33286.75999999999</v>
+        <v>32632.12</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.5910164764280185</v>
+        <v>0.5990598238091143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-23 17:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0</v>
+        <v>312.26</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>0</v>
@@ -1617,10 +1617,10 @@
         <v>0</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>0</v>
+        <v>457.23</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>933.8099999999999</v>
+        <v>1434.19</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -4581,52 +4581,52 @@
     <row r="69">
       <c r="C69" s="4" t="inlineStr">
         <is>
+          <t>1 de 67</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>3 de 67</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>1 de 67</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
           <t>0 de 67</t>
         </is>
       </c>
-      <c r="D69" s="4" t="inlineStr">
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>0 de 67</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>6 de 67</t>
+        </is>
+      </c>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>7 de 67</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr">
+        <is>
+          <t>0 de 67</t>
+        </is>
+      </c>
+      <c r="K69" s="4" t="inlineStr">
         <is>
           <t>3 de 67</t>
         </is>
       </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>1 de 67</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="inlineStr">
-        <is>
-          <t>0 de 67</t>
-        </is>
-      </c>
-      <c r="G69" s="4" t="inlineStr">
-        <is>
-          <t>0 de 67</t>
-        </is>
-      </c>
-      <c r="H69" s="4" t="inlineStr">
-        <is>
-          <t>6 de 67</t>
-        </is>
-      </c>
-      <c r="I69" s="4" t="inlineStr">
-        <is>
-          <t>7 de 67</t>
-        </is>
-      </c>
-      <c r="J69" s="4" t="inlineStr">
-        <is>
-          <t>0 de 67</t>
-        </is>
-      </c>
-      <c r="K69" s="4" t="inlineStr">
-        <is>
-          <t>3 de 67</t>
-        </is>
-      </c>
       <c r="L69" s="4" t="inlineStr">
         <is>
-          <t>8 de 67</t>
+          <t>9 de 67</t>
         </is>
       </c>
       <c r="M69" s="4" t="inlineStr">
@@ -5011,7 +5011,7 @@
         <v>1205.88</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>1872.91</v>
+        <v>2185.17</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>1500</v>
@@ -5065,7 +5065,7 @@
         <v>4090.91</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>933.8099999999999</v>
+        <v>1891.42</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>2000</v>
@@ -6000,7 +6000,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>48756.88</v>
+        <v>50026.75</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6023,7 +6023,7 @@
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
@@ -6075,13 +6075,13 @@
         <v>536</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0</v>
+        <v>312.26</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>536</v>
+        <v>223.74</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0</v>
+        <v>0.5825746268656716</v>
       </c>
     </row>
     <row r="3">
@@ -6339,13 +6339,13 @@
         <v>2534</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>6549.96</v>
+        <v>7007.19</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-4015.96</v>
+        <v>-4473.19</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>2.584830307813733</v>
+        <v>2.765268350434096</v>
       </c>
     </row>
     <row r="14">
@@ -6363,13 +6363,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>24116.62</v>
+        <v>24617</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>34005.38</v>
+        <v>33505</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.414931007191769</v>
+        <v>0.4235401397061354</v>
       </c>
     </row>
     <row r="15">
@@ -6406,13 +6406,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>48756.88</v>
+        <v>50026.75</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>32632.12</v>
+        <v>31362.25</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.5990598238091143</v>
+        <v>0.6146623008023198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-24 08:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2940,7 +2940,7 @@
         <v>1480.89</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>7296.12</v>
+        <v>7275.4</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -5443,7 +5443,7 @@
         <v>6566.73</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>9972.26</v>
+        <v>9951.540000000001</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>6000</v>
@@ -6000,7 +6000,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>50026.75</v>
+        <v>50006.03</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6023,7 +6023,7 @@
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
@@ -6363,13 +6363,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>24617</v>
+        <v>24596.28</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>33505</v>
+        <v>33525.72</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.4235401397061354</v>
+        <v>0.4231836481882936</v>
       </c>
     </row>
     <row r="15">
@@ -6406,13 +6406,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>50026.75</v>
+        <v>50006.03</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>31362.25</v>
+        <v>31382.97</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.6146623008023198</v>
+        <v>0.6144077209450909</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-24 09:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2877,7 +2877,7 @@
         <v>-43.43</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>0</v>
+        <v>2045.75</v>
       </c>
       <c r="M40" s="2" t="n">
         <v>0</v>
@@ -3780,7 +3780,7 @@
         <v>0</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>0</v>
+        <v>642.16</v>
       </c>
       <c r="N55" s="2" t="n">
         <v>0</v>
@@ -4626,12 +4626,12 @@
       </c>
       <c r="L69" s="4" t="inlineStr">
         <is>
-          <t>9 de 67</t>
+          <t>10 de 67</t>
         </is>
       </c>
       <c r="M69" s="4" t="inlineStr">
         <is>
-          <t>14 de 67</t>
+          <t>15 de 67</t>
         </is>
       </c>
       <c r="N69" s="4" t="inlineStr">
@@ -5416,7 +5416,7 @@
         <v>10443.14</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>-43.43</v>
+        <v>2002.32</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>0</v>
@@ -5740,7 +5740,7 @@
         <v>0</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0</v>
+        <v>642.16</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>0</v>
@@ -6000,7 +6000,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>50006.03</v>
+        <v>52693.94</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6339,13 +6339,13 @@
         <v>2534</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>7007.19</v>
+        <v>9052.940000000001</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-4473.19</v>
+        <v>-6518.940000000001</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>2.765268350434096</v>
+        <v>3.572588792423047</v>
       </c>
     </row>
     <row r="14">
@@ -6363,13 +6363,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>24596.28</v>
+        <v>25238.44</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>33525.72</v>
+        <v>32883.56</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.4231836481882936</v>
+        <v>0.4342321324111352</v>
       </c>
     </row>
     <row r="15">
@@ -6406,13 +6406,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>50006.03</v>
+        <v>52693.94</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>31382.97</v>
+        <v>28695.06</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.6144077209450909</v>
+        <v>0.6474331912174864</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-24 15:30:18
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2937,7 +2937,7 @@
         <v>0</v>
       </c>
       <c r="L41" s="2" t="n">
-        <v>1480.89</v>
+        <v>2299.19</v>
       </c>
       <c r="M41" s="2" t="n">
         <v>7275.4</v>
@@ -3780,7 +3780,7 @@
         <v>0</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>642.16</v>
+        <v>1544</v>
       </c>
       <c r="N55" s="2" t="n">
         <v>0</v>
@@ -5443,7 +5443,7 @@
         <v>6566.73</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>9951.540000000001</v>
+        <v>10769.84</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>6000</v>
@@ -5740,7 +5740,7 @@
         <v>0</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>642.16</v>
+        <v>1544</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>0</v>
@@ -6000,7 +6000,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>52693.94</v>
+        <v>54414.08</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6339,13 +6339,13 @@
         <v>2534</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>9052.940000000001</v>
+        <v>9871.24</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-6518.940000000001</v>
+        <v>-7337.24</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>3.572588792423047</v>
+        <v>3.895516969218626</v>
       </c>
     </row>
     <row r="14">
@@ -6363,13 +6363,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>25238.44</v>
+        <v>26140.28</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>32883.56</v>
+        <v>31981.72</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.4342321324111352</v>
+        <v>0.4497484601355768</v>
       </c>
     </row>
     <row r="15">
@@ -6406,13 +6406,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>52693.94</v>
+        <v>54414.08</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>28695.06</v>
+        <v>26974.92</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.6474331912174864</v>
+        <v>0.6685679883030876</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-24 17:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -1740,7 +1740,7 @@
         <v>0</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>2243.53</v>
+        <v>4297.4</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
@@ -5092,7 +5092,7 @@
         <v>0</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>2243.53</v>
+        <v>4297.4</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>2000</v>
@@ -6000,7 +6000,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>54414.08</v>
+        <v>56467.95</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6363,13 +6363,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>26140.28</v>
+        <v>28194.15</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>31981.72</v>
+        <v>29927.85</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.4497484601355768</v>
+        <v>0.4850856818416435</v>
       </c>
     </row>
     <row r="15">
@@ -6406,13 +6406,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>54414.08</v>
+        <v>56467.95</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>26974.92</v>
+        <v>24921.05</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.6685679883030876</v>
+        <v>0.6938032166508988</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-25 17:30:18
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2940,7 +2940,7 @@
         <v>2299.19</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>7275.4</v>
+        <v>7254.68</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -5443,7 +5443,7 @@
         <v>6566.73</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>11528.12</v>
+        <v>11507.4</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>6000</v>
@@ -6000,7 +6000,7 @@
         <v>61257.37</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>57226.23</v>
+        <v>57205.51</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>82000</v>
@@ -6363,13 +6363,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>28194.15</v>
+        <v>28173.43</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>29927.85</v>
+        <v>29948.57</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.4850856818416435</v>
+        <v>0.4847291903238017</v>
       </c>
     </row>
     <row r="15">
@@ -6406,13 +6406,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>57226.23</v>
+        <v>57205.51</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>24162.77</v>
+        <v>24183.49</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.7031199547850447</v>
+        <v>0.7028653749278159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-28 08:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -4671,7 +4671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5106,7 +5106,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ECUASERVIMUNDO S.A.</t>
+          <t>CONSTRUDISMAT S.A. HERNANDEZ ESTEVES NORA ESPERANZA</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -5116,7 +5116,7 @@
         <v>0</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>250.17</v>
+        <v>0</v>
       </c>
       <c r="F16" s="2" t="n">
         <v>0</v>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ELITE SUPPLY ELISU S.A.S.</t>
+          <t>ECUASERVIMUNDO S.A.</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -5143,13 +5143,13 @@
         <v>0</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0</v>
+        <v>250.17</v>
       </c>
       <c r="F17" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -5160,7 +5160,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ESCOBAR SAMANIEGO VICENTE</t>
+          <t>ELITE SUPPLY ELISU S.A.S.</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -5173,10 +5173,10 @@
         <v>0</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>1728.65</v>
+        <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>3000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="19">
@@ -5187,23 +5187,23 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ESCOBAR SANCHEZ INGRIN MAGALI</t>
+          <t>ESCOBAR SAMANIEGO VICENTE</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>5238.16</v>
+        <v>0</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>3117.5</v>
+        <v>0</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0</v>
+        <v>1728.65</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="20">
@@ -5214,23 +5214,23 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FERREZACA (FERRETERIA ZAMBRANO CAMPOVERDE) S.A.S.</t>
+          <t>ESCOBAR SANCHEZ INGRIN MAGALI</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>255.54</v>
+        <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>1148.2</v>
+        <v>5238.16</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0</v>
+        <v>3117.5</v>
       </c>
       <c r="F20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>1500</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="21">
@@ -5241,14 +5241,14 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FERROCENTER CONSTRUCCION ACABADOS FERCONAC SAS</t>
+          <t>FERREZACA (FERRETERIA ZAMBRANO CAMPOVERDE) S.A.S.</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1132.19</v>
+        <v>255.54</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0</v>
+        <v>1148.2</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>0</v>
@@ -5257,7 +5257,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>3000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="22">
@@ -5268,23 +5268,23 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>GENEAL S.A.</t>
+          <t>FERROCENTER CONSTRUCCION ACABADOS FERCONAC SAS</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>308.61</v>
+        <v>1132.19</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>719.61</v>
+        <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>3084.74</v>
+        <v>0</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="23">
@@ -5295,20 +5295,20 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GLOBALMATCH S.A.S.</t>
+          <t>GENEAL S.A.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>923.37</v>
+        <v>308.61</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>499.66</v>
+        <v>0</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>178.5</v>
+        <v>719.61</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0</v>
+        <v>3084.74</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>2000</v>
@@ -5322,23 +5322,23 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>GOYA CASTRO CARLOS ALBERTO</t>
+          <t>GLOBALMATCH S.A.S.</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>740.08</v>
+        <v>923.37</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>379.14</v>
+        <v>499.66</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>1591.53</v>
+        <v>178.5</v>
       </c>
       <c r="F24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="25">
@@ -5349,23 +5349,23 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>INTRIAGO ALVARADO BRENDA ALEJANDRA</t>
+          <t>GOYA CASTRO CARLOS ALBERTO</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>5187.69</v>
+        <v>740.08</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>17576.46</v>
+        <v>379.14</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>7198.47</v>
+        <v>1591.53</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>3162.84</v>
+        <v>0</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="26">
@@ -5376,23 +5376,23 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>JACOME MONCAYO JAVIER ALFONSO</t>
+          <t>INTRIAGO ALVARADO BRENDA ALEJANDRA</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>5709.49</v>
+        <v>5187.69</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>-52.9</v>
+        <v>17576.46</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>5275.56</v>
+        <v>7198.47</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>4433</v>
+        <v>3162.84</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -5403,23 +5403,23 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>JOWIN SA</t>
+          <t>JACOME MONCAYO JAVIER ALFONSO</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>751.88</v>
+        <v>5709.49</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>6023.41</v>
+        <v>-52.9</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>10443.14</v>
+        <v>5275.56</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>2002.32</v>
+        <v>4433</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="28">
@@ -5430,23 +5430,23 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MAD&amp;DECO S.A.</t>
+          <t>JOWIN SA</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>4315.06</v>
+        <v>751.88</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>8512.780000000001</v>
+        <v>6023.41</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>6566.73</v>
+        <v>10443.14</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>11507.4</v>
+        <v>2002.32</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>6000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -5457,23 +5457,23 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MAJACSA S.A.</t>
+          <t>MAD&amp;DECO S.A.</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1149.87</v>
+        <v>4315.06</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0</v>
+        <v>8512.780000000001</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0</v>
+        <v>6566.73</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0</v>
+        <v>11507.4</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>1500</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="30">
@@ -5484,11 +5484,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MEGAMETALES S.A.</t>
+          <t>MAJACSA S.A.</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0</v>
+        <v>1149.87</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>0</v>
@@ -5497,10 +5497,10 @@
         <v>0</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>1324.05</v>
+        <v>0</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>5000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="31">
@@ -5511,23 +5511,23 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MONCAYO PINCAY JOSE GREGORIO</t>
+          <t>MEGAMETALES S.A.</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>261.27</v>
+        <v>0</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0</v>
+        <v>1324.05</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="32">
@@ -5538,20 +5538,20 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PEREZ NARANJO JOYCE LORENA</t>
+          <t>MONCAYO PINCAY JOSE GREGORIO</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>2959.75</v>
+        <v>261.27</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>379.14</v>
+        <v>0</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>379.64</v>
+        <v>0</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>0</v>
@@ -5565,23 +5565,23 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PERUCCI .S.A</t>
+          <t>PEREZ NARANJO JOYCE LORENA</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0</v>
+        <v>2959.75</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0</v>
+        <v>379.14</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>0</v>
+        <v>379.64</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -5592,11 +5592,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PIEDRA VALDEZ GENESIS DAYANNA</t>
+          <t>PERUCCI .S.A</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>84.55</v>
+        <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>0</v>
@@ -5605,10 +5605,10 @@
         <v>0</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>59.62</v>
+        <v>0</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="35">
@@ -5619,23 +5619,23 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>QUIROZ PEÑAFIEL DIANA ISABEL</t>
+          <t>PIEDRA VALDEZ GENESIS DAYANNA</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>1268.07</v>
+        <v>84.55</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>672.05</v>
+        <v>0</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>831.75</v>
+        <v>0</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0</v>
+        <v>59.62</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -5646,23 +5646,23 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>RAMOS BARRENO LIZ TAMARA</t>
+          <t>QUIROZ PEÑAFIEL DIANA ISABEL</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0</v>
+        <v>1268.07</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>3129.2</v>
+        <v>672.05</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>4677.09</v>
+        <v>831.75</v>
       </c>
       <c r="F36" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="37">
@@ -5673,23 +5673,23 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>RAMOS RODRIGUEZ ADRIANA CAROLINA</t>
+          <t>RAMOS BARRENO LIZ TAMARA</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>192.35</v>
+        <v>0</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>-156.11</v>
+        <v>3129.2</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>3828.29</v>
+        <v>4677.09</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>-454.9</v>
+        <v>0</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>1500</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="38">
@@ -5700,20 +5700,20 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>RIVERA CANTOS MARTHA JACQUELIN</t>
+          <t>RAMOS RODRIGUEZ ADRIANA CAROLINA</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>0</v>
+        <v>192.35</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0</v>
+        <v>-156.11</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0</v>
+        <v>3828.29</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>2194.33</v>
+        <v>-454.9</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>1500</v>
@@ -5727,23 +5727,23 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>RUIZ PINEDA LUIS ALFREDO</t>
+          <t>RIVERA CANTOS MARTHA JACQUELIN</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>342.23</v>
+        <v>0</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>2526.87</v>
+        <v>0</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>1544</v>
+        <v>2194.33</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="40">
@@ -5754,23 +5754,23 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>SALAZAR BALLADARES MARIA ANGELICA</t>
+          <t>RUIZ PINEDA LUIS ALFREDO</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>3136.9</v>
+        <v>342.23</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>4598.29</v>
+        <v>2526.87</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>24.06</v>
+        <v>0</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>3208.32</v>
+        <v>1544</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -5781,23 +5781,23 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SANCHEZ CORREA MARCO EDUARDO</t>
+          <t>SALAZAR BALLADARES MARIA ANGELICA</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>3242.94</v>
+        <v>3136.9</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>794.33</v>
+        <v>4598.29</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>2665.26</v>
+        <v>24.06</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>2736.22</v>
+        <v>3208.32</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="42">
@@ -5808,23 +5808,23 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SERVICERAMICAS S.A.S.</t>
+          <t>SANCHEZ CORREA MARCO EDUARDO</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>31.3</v>
+        <v>3242.94</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>497.4</v>
+        <v>794.33</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>1696.95</v>
+        <v>2665.26</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>1238.73</v>
+        <v>2736.22</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="43">
@@ -5835,23 +5835,23 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SISA GUANO CARLOS ALBERTO</t>
+          <t>SERVICERAMICAS S.A.S.</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>812.16</v>
+        <v>31.3</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>-768.3</v>
+        <v>497.4</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>1199.43</v>
+        <v>1696.95</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0</v>
+        <v>1238.73</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="44">
@@ -5862,23 +5862,23 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SUSANDECORATIONS S.A.S.</t>
+          <t>SISA GUANO CARLOS ALBERTO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>0</v>
+        <v>812.16</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>0</v>
+        <v>-768.3</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>0</v>
+        <v>1199.43</v>
       </c>
       <c r="F44" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="45">
@@ -5889,11 +5889,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>TAPIA BALLADARES LORENA ELIZABETH</t>
+          <t>SUSANDECORATIONS S.A.S.</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>2549.83</v>
+        <v>0</v>
       </c>
       <c r="D45" s="2" t="n">
         <v>0</v>
@@ -5902,10 +5902,10 @@
         <v>0</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>3897.51</v>
+        <v>0</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -5916,11 +5916,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>TAPIA TAPIA ANGEL GUSTAVO</t>
+          <t>TAPIA BALLADARES LORENA ELIZABETH</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>2036.39</v>
+        <v>2549.83</v>
       </c>
       <c r="D46" s="2" t="n">
         <v>0</v>
@@ -5929,10 +5929,10 @@
         <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>0</v>
+        <v>3897.51</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="47">
@@ -5943,14 +5943,14 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>TRANSCASH S.A.</t>
+          <t>TAPIA TAPIA ANGEL GUSTAVO</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>0</v>
+        <v>2036.39</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>1375.93</v>
+        <v>0</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>0</v>
@@ -5959,7 +5959,7 @@
         <v>0</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="48">
@@ -5970,39 +5970,66 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
+          <t>TRANSCASH S.A.</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>1375.93</v>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>CASTRO ALCIVAR EDA MARIA</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
           <t>VIZUETA CAZORLA SUSANA JOHANNA</t>
         </is>
       </c>
-      <c r="C48" s="2" t="n">
+      <c r="C49" s="2" t="n">
         <v>595.03</v>
       </c>
-      <c r="D48" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E48" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F48" s="2" t="n">
+      <c r="D49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="2" t="n">
         <v>891.11</v>
       </c>
-      <c r="G48" s="2" t="n">
+      <c r="G49" s="2" t="n">
         <v>1000</v>
       </c>
     </row>
-    <row r="49">
-      <c r="C49" s="6" t="n">
+    <row r="50">
+      <c r="C50" s="6" t="n">
         <v>48353.56</v>
       </c>
-      <c r="D49" s="6" t="n">
+      <c r="D50" s="6" t="n">
         <v>71913.73</v>
       </c>
-      <c r="E49" s="6" t="n">
+      <c r="E50" s="6" t="n">
         <v>61257.37</v>
       </c>
-      <c r="F49" s="6" t="n">
+      <c r="F50" s="6" t="n">
         <v>57205.51</v>
       </c>
-      <c r="G49" s="6" t="n">
+      <c r="G50" s="6" t="n">
         <v>82000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-09-28 10:30:19
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -3213,7 +3213,7 @@
         <v>0</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>0</v>
+        <v>758.28</v>
       </c>
       <c r="E46" s="2" t="n">
         <v>0</v>
@@ -3228,7 +3228,7 @@
         <v>0</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>0</v>
+        <v>174.74</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0</v>
@@ -3888,7 +3888,7 @@
         <v>0</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>1499.57</v>
+        <v>1577.63</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0</v>
@@ -4586,7 +4586,7 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>3 de 67</t>
+          <t>4 de 67</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
@@ -4611,7 +4611,7 @@
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>7 de 67</t>
+          <t>8 de 67</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr">
@@ -5578,7 +5578,7 @@
         <v>379.14</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>379.64</v>
+        <v>1312.66</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>0</v>
@@ -5821,7 +5821,7 @@
         <v>2665.26</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>2736.22</v>
+        <v>2814.28</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>3000</v>
@@ -6027,7 +6027,7 @@
         <v>61257.37</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>57205.51</v>
+        <v>58216.59</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>82000</v>
@@ -6126,13 +6126,13 @@
         <v>7842</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2898.82</v>
+        <v>3657.1</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>4943.18</v>
+        <v>4184.9</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.3696531497067075</v>
+        <v>0.466347870441214</v>
       </c>
     </row>
     <row r="4">
@@ -6246,13 +6246,13 @@
         <v>1676</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>4499.36</v>
+        <v>4752.16</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-2823.36</v>
+        <v>-3076.16</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>2.684582338902148</v>
+        <v>2.835417661097852</v>
       </c>
     </row>
     <row r="9">
@@ -6433,13 +6433,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>57205.51</v>
+        <v>58216.59</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>24183.49</v>
+        <v>23172.41</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.7028653749278159</v>
+        <v>0.7152881839069162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-28 15:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2814,13 +2814,13 @@
         <v>0</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>0</v>
+        <v>744.48</v>
       </c>
       <c r="L39" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>0</v>
+        <v>5577.02</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>0</v>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="K69" s="4" t="inlineStr">
         <is>
-          <t>3 de 67</t>
+          <t>4 de 67</t>
         </is>
       </c>
       <c r="L69" s="4" t="inlineStr">
@@ -4631,7 +4631,7 @@
       </c>
       <c r="M69" s="4" t="inlineStr">
         <is>
-          <t>15 de 67</t>
+          <t>16 de 67</t>
         </is>
       </c>
       <c r="N69" s="4" t="inlineStr">
@@ -5416,7 +5416,7 @@
         <v>5275.56</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>4433</v>
+        <v>10754.5</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>5000</v>
@@ -6027,7 +6027,7 @@
         <v>61257.37</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>58216.59</v>
+        <v>64538.09</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>82000</v>
@@ -6318,13 +6318,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>2870.08</v>
+        <v>3614.56</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-2142.08</v>
+        <v>-2886.56</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>3.942417582417582</v>
+        <v>4.965054945054945</v>
       </c>
     </row>
     <row r="12">
@@ -6390,13 +6390,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>28173.43</v>
+        <v>33750.45</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>29948.57</v>
+        <v>24371.55</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.4847291903238017</v>
+        <v>0.5806828739547847</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>58216.59</v>
+        <v>64538.09</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>23172.41</v>
+        <v>16850.91</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.7152881839069162</v>
+        <v>0.7929583850397474</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-29 09:30:18
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2736,7 +2736,7 @@
         <v>1696.4</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0</v>
+        <v>64.81999999999999</v>
       </c>
       <c r="F38" s="2" t="n">
         <v>0</v>
@@ -3714,7 +3714,7 @@
         <v>0</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>2124.4</v>
+        <v>2085.7</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
@@ -4128,7 +4128,7 @@
         <v>0</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>0</v>
+        <v>426.43</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0</v>
@@ -4591,7 +4591,7 @@
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>1 de 67</t>
+          <t>2 de 67</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr">
@@ -4611,7 +4611,7 @@
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>8 de 67</t>
+          <t>9 de 67</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr">
@@ -5389,7 +5389,7 @@
         <v>7198.47</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>3162.84</v>
+        <v>3227.66</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>0</v>
@@ -5740,7 +5740,7 @@
         <v>0</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>2194.33</v>
+        <v>2155.63</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>1500</v>
@@ -5875,7 +5875,7 @@
         <v>1199.43</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0</v>
+        <v>426.43</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>1500</v>
@@ -6027,7 +6027,7 @@
         <v>61257.37</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>64538.09</v>
+        <v>64990.64</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>82000</v>
@@ -6174,13 +6174,13 @@
         <v>199.5</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>194.46</v>
+        <v>259.28</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5.039999999999992</v>
+        <v>-59.77999999999997</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0.9747368421052632</v>
+        <v>1.299649122807017</v>
       </c>
     </row>
     <row r="6">
@@ -6246,13 +6246,13 @@
         <v>1676</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>4752.16</v>
+        <v>5178.59</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-3076.16</v>
+        <v>-3502.59</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>2.835417661097852</v>
+        <v>3.089850835322196</v>
       </c>
     </row>
     <row r="9">
@@ -6318,13 +6318,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>3614.56</v>
+        <v>3575.86</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-2886.56</v>
+        <v>-2847.86</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>4.965054945054945</v>
+        <v>4.911895604395604</v>
       </c>
     </row>
     <row r="12">
@@ -6433,13 +6433,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>64538.09</v>
+        <v>64990.64</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>16850.91</v>
+        <v>16398.36</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.7929583850397474</v>
+        <v>0.7985187187457764</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-29 10:30:19
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -3234,7 +3234,7 @@
         <v>0</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>379.64</v>
+        <v>990.01</v>
       </c>
       <c r="L46" s="2" t="n">
         <v>0</v>
@@ -5578,7 +5578,7 @@
         <v>379.14</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>1312.66</v>
+        <v>1923.03</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>0</v>
@@ -6027,7 +6027,7 @@
         <v>61257.37</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>64990.64</v>
+        <v>65601.00999999999</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>82000</v>
@@ -6318,13 +6318,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>3575.86</v>
+        <v>4186.23</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-2847.86</v>
+        <v>-3458.23</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>4.911895604395604</v>
+        <v>5.750315934065934</v>
       </c>
     </row>
     <row r="12">
@@ -6433,13 +6433,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>64990.64</v>
+        <v>65601.00999999999</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>16398.36</v>
+        <v>15787.99</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.7985187187457764</v>
+        <v>0.8060181351288257</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-29 14:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -4020,7 +4020,7 @@
         <v>1219.77</v>
       </c>
       <c r="M59" s="2" t="n">
-        <v>18.96</v>
+        <v>1303.28</v>
       </c>
       <c r="N59" s="2" t="n">
         <v>0</v>
@@ -5848,7 +5848,7 @@
         <v>1696.95</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>1238.73</v>
+        <v>2523.05</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>2000</v>
@@ -6027,7 +6027,7 @@
         <v>61257.37</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>65601.00999999999</v>
+        <v>66885.33</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>82000</v>
@@ -6390,13 +6390,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>33750.45</v>
+        <v>35034.77</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>24371.55</v>
+        <v>23087.23</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.5806828739547847</v>
+        <v>0.6027798424004679</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>65601.00999999999</v>
+        <v>66885.32999999999</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>15787.99</v>
+        <v>14503.67</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.8060181351288257</v>
+        <v>0.8217981545417684</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-29 16:30:19
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2940,7 +2940,7 @@
         <v>2299.19</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>7254.68</v>
+        <v>7275.4</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -5470,7 +5470,7 @@
         <v>6566.73</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>11507.4</v>
+        <v>11528.12</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>6000</v>
@@ -6027,7 +6027,7 @@
         <v>61257.37</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>66885.33</v>
+        <v>66906.05</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>82000</v>
@@ -6390,13 +6390,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>35034.77</v>
+        <v>35055.49</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>23087.23</v>
+        <v>23066.51</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.6027798424004679</v>
+        <v>0.6031363339183097</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>66885.32999999999</v>
+        <v>66906.04999999999</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>14503.67</v>
+        <v>14482.95</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.8217981545417684</v>
+        <v>0.8220527343989973</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-30 08:30:18
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2760,7 +2760,7 @@
         <v>654.64</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>0</v>
+        <v>3837.05</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -2940,7 +2940,7 @@
         <v>2299.19</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>7275.4</v>
+        <v>9046.700000000001</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -3840,7 +3840,7 @@
         <v>423.26</v>
       </c>
       <c r="M56" s="2" t="n">
-        <v>2026.04</v>
+        <v>3634.34</v>
       </c>
       <c r="N56" s="2" t="n">
         <v>0</v>
@@ -4554,7 +4554,7 @@
         <v>0</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>446.69</v>
+        <v>744.49</v>
       </c>
       <c r="L68" s="2" t="n">
         <v>0</v>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="M69" s="4" t="inlineStr">
         <is>
-          <t>16 de 67</t>
+          <t>17 de 67</t>
         </is>
       </c>
       <c r="N69" s="4" t="inlineStr">
@@ -5389,7 +5389,7 @@
         <v>7198.47</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>3227.66</v>
+        <v>7064.71</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>0</v>
@@ -5470,7 +5470,7 @@
         <v>6566.73</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>11528.12</v>
+        <v>13299.42</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>6000</v>
@@ -5794,7 +5794,7 @@
         <v>24.06</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>3208.32</v>
+        <v>4816.62</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>4000</v>
@@ -6010,7 +6010,7 @@
         <v>0</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>891.11</v>
+        <v>1286.02</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>1000</v>
@@ -6027,7 +6027,7 @@
         <v>61257.37</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>66906.05</v>
+        <v>74517.61</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>82000</v>
@@ -6318,13 +6318,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>4186.23</v>
+        <v>4484.03</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-3458.23</v>
+        <v>-3756.03</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>5.750315934065934</v>
+        <v>6.159381868131867</v>
       </c>
     </row>
     <row r="12">
@@ -6342,13 +6342,13 @@
         <v>350</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0</v>
+        <v>97.11</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>350</v>
+        <v>252.89</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0</v>
+        <v>0.2774571428571428</v>
       </c>
     </row>
     <row r="13">
@@ -6390,13 +6390,13 @@
         <v>58122</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>35055.49</v>
+        <v>42272.14</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>23066.51</v>
+        <v>15849.86</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.6031363339183097</v>
+        <v>0.7273001617287774</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>66906.04999999999</v>
+        <v>74517.61</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>14482.95</v>
+        <v>6871.389999999998</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.8220527343989973</v>
+        <v>0.9155734804457605</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-30 09:30:22
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2865,10 +2865,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>0</v>
+        <v>2268.09</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>0</v>
+        <v>286.21</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0</v>
@@ -4606,12 +4606,12 @@
       </c>
       <c r="H69" s="4" t="inlineStr">
         <is>
-          <t>6 de 67</t>
+          <t>7 de 67</t>
         </is>
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>9 de 67</t>
+          <t>10 de 67</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr">
@@ -5443,7 +5443,7 @@
         <v>10443.14</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>2002.32</v>
+        <v>4556.62</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>0</v>
@@ -6027,7 +6027,7 @@
         <v>61257.37</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>74517.61</v>
+        <v>77071.91</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>82000</v>
@@ -6222,13 +6222,13 @@
         <v>2450</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>8368.780000000001</v>
+        <v>10636.87</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-5918.780000000001</v>
+        <v>-8186.870000000001</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>3.415828571428572</v>
+        <v>4.341579591836735</v>
       </c>
     </row>
     <row r="8">
@@ -6246,13 +6246,13 @@
         <v>1676</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>5178.59</v>
+        <v>5464.8</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-3502.59</v>
+        <v>-3788.8</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>3.089850835322196</v>
+        <v>3.260620525059666</v>
       </c>
     </row>
     <row r="9">
@@ -6433,13 +6433,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>74517.61</v>
+        <v>77071.91</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>6871.389999999998</v>
+        <v>4317.089999999998</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.9155734804457605</v>
+        <v>0.9469573283858999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-30 15:30:18
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2865,7 +2865,7 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>2268.09</v>
+        <v>4181.43</v>
       </c>
       <c r="I40" s="2" t="n">
         <v>286.21</v>
@@ -3234,7 +3234,7 @@
         <v>0</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>990.01</v>
+        <v>1037.39</v>
       </c>
       <c r="L46" s="2" t="n">
         <v>0</v>
@@ -5443,7 +5443,7 @@
         <v>10443.14</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>4556.62</v>
+        <v>6469.96</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>0</v>
@@ -5578,7 +5578,7 @@
         <v>379.14</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>1923.03</v>
+        <v>1970.41</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>0</v>
@@ -6027,7 +6027,7 @@
         <v>61257.37</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>77071.91</v>
+        <v>79032.63</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>82000</v>
@@ -6222,13 +6222,13 @@
         <v>2450</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>10636.87</v>
+        <v>12550.21</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-8186.870000000001</v>
+        <v>-10100.21</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>4.341579591836735</v>
+        <v>5.122534693877551</v>
       </c>
     </row>
     <row r="8">
@@ -6318,13 +6318,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>4484.03</v>
+        <v>4531.41</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-3756.03</v>
+        <v>-3803.41</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>6.159381868131867</v>
+        <v>6.224464285714285</v>
       </c>
     </row>
     <row r="12">
@@ -6433,13 +6433,13 @@
         <v>81389</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>77071.91</v>
+        <v>79032.63</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>4317.089999999998</v>
+        <v>2356.369999999999</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.9469573283858999</v>
+        <v>0.9710480531767193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-01 09:30:30
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2634,7 +2634,7 @@
         <v>0</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>0</v>
+        <v>223.34</v>
       </c>
       <c r="L36" s="2" t="n">
         <v>0</v>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="K69" s="4" t="inlineStr">
         <is>
-          <t>0 de 67</t>
+          <t>1 de 67</t>
         </is>
       </c>
       <c r="L69" s="4" t="inlineStr">
@@ -5362,7 +5362,7 @@
         <v>268.27</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0</v>
+        <v>223.34</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>1000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>0</v>
+        <v>223.34</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>82000</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-01 14:30:15
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -1500,7 +1500,7 @@
         <v>0</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>0</v>
+        <v>72.03</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
@@ -1620,7 +1620,7 @@
         <v>0</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>0</v>
+        <v>147.07</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="M69" s="4" t="inlineStr">
         <is>
-          <t>0 de 67</t>
+          <t>2 de 67</t>
         </is>
       </c>
       <c r="N69" s="4" t="inlineStr">
@@ -5011,7 +5011,7 @@
         <v>2185.17</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0</v>
+        <v>72.03</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>1500</v>
@@ -5065,7 +5065,7 @@
         <v>2184.08</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>147.07</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>2000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>223.34</v>
+        <v>442.44</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>82000</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-02 12:30:14
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -1740,7 +1740,7 @@
         <v>0</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>0</v>
+        <v>2738.84</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="M69" s="4" t="inlineStr">
         <is>
-          <t>2 de 67</t>
+          <t>3 de 67</t>
         </is>
       </c>
       <c r="N69" s="4" t="inlineStr">
@@ -5092,7 +5092,7 @@
         <v>4297.4</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0</v>
+        <v>2738.84</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>2000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>442.44</v>
+        <v>3181.28</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>82000</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-02 17:30:15
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -3234,7 +3234,7 @@
         <v>0</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>0</v>
+        <v>-47.38</v>
       </c>
       <c r="L46" s="2" t="n">
         <v>0</v>
@@ -5578,7 +5578,7 @@
         <v>1970.41</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>0</v>
+        <v>-47.38</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>0</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>3181.28</v>
+        <v>3133.9</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>82000</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-05 12:08:43
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -4852,7 +4852,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="7">
@@ -4879,7 +4879,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>5000</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="8">
@@ -4906,7 +4906,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -4933,7 +4933,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="10">
@@ -4960,7 +4960,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -4987,7 +4987,7 @@
         <v>0</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="12">
@@ -5095,7 +5095,7 @@
         <v>2738.84</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>2000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="16">
@@ -5176,7 +5176,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -5230,7 +5230,7 @@
         <v>0</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="21">
@@ -5311,7 +5311,7 @@
         <v>0</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="24">
@@ -5392,7 +5392,7 @@
         <v>0</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="27">
@@ -5473,7 +5473,7 @@
         <v>0</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>6000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="30">
@@ -5527,7 +5527,7 @@
         <v>0</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -5581,7 +5581,7 @@
         <v>-47.38</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="34">
@@ -5608,7 +5608,7 @@
         <v>0</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -5635,7 +5635,7 @@
         <v>0</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="36">
@@ -5662,7 +5662,7 @@
         <v>0</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -5689,7 +5689,7 @@
         <v>0</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>3000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="38">
@@ -5716,7 +5716,7 @@
         <v>0</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="39">
@@ -5770,7 +5770,7 @@
         <v>0</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="41">
@@ -5797,7 +5797,7 @@
         <v>0</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>4000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="42">
@@ -5824,7 +5824,7 @@
         <v>0</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="43">
@@ -5932,7 +5932,7 @@
         <v>0</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="47">
@@ -5959,7 +5959,7 @@
         <v>0</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -6013,7 +6013,7 @@
         <v>0</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="50">
@@ -6030,7 +6030,7 @@
         <v>3133.9</v>
       </c>
       <c r="G50" s="6" t="n">
-        <v>82000</v>
+        <v>81531</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-06 08:30:14
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -4233,7 +4233,7 @@
         <v>0</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>0</v>
+        <v>129.99</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>0</v>
@@ -4586,7 +4586,7 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>0 de 67</t>
+          <t>1 de 67</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
@@ -5929,7 +5929,7 @@
         <v>3897.51</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>0</v>
+        <v>129.99</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>3000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>3133.9</v>
+        <v>3263.89</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-06 09:30:14
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -5254,7 +5254,7 @@
         <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0</v>
+        <v>34.48</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>1500</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>3263.89</v>
+        <v>3298.37</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-06 14:30:14
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -5713,7 +5713,7 @@
         <v>-454.9</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0</v>
+        <v>2676.24</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>2000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>3298.37</v>
+        <v>5974.61</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-07 11:30:14
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -5929,7 +5929,7 @@
         <v>3897.51</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>129.99</v>
+        <v>164.47</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>3000</v>
@@ -6010,7 +6010,7 @@
         <v>1286.02</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>0</v>
+        <v>34.48</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>1500</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>8465.65</v>
+        <v>8534.610000000001</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-08 09:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -5389,7 +5389,7 @@
         <v>7064.71</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0</v>
+        <v>3008.2</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>5000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>10738.81</v>
+        <v>13747.01</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-12 09:30:15
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -5200,7 +5200,7 @@
         <v>1728.65</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0</v>
+        <v>34.48</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>3000</v>
@@ -5713,7 +5713,7 @@
         <v>-454.9</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>4880.44</v>
+        <v>7474.15</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>2000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>13747.01</v>
+        <v>16375.2</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-12 11:30:15
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -3540,7 +3540,7 @@
         <v>0</v>
       </c>
       <c r="M51" s="2" t="n">
-        <v>0</v>
+        <v>33.12</v>
       </c>
       <c r="N51" s="2" t="n">
         <v>0</v>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="M69" s="4" t="inlineStr">
         <is>
-          <t>4 de 67</t>
+          <t>5 de 67</t>
         </is>
       </c>
       <c r="N69" s="4" t="inlineStr">
@@ -5686,7 +5686,7 @@
         <v>4313.71</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0</v>
+        <v>33.12</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>5000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>16375.2</v>
+        <v>16408.32</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-12 13:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2940,7 +2940,7 @@
         <v>0</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>0</v>
+        <v>-18.65</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -5470,7 +5470,7 @@
         <v>13299.42</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0</v>
+        <v>-18.65</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>5000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>16408.32</v>
+        <v>16389.67</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-13 09:30:19
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -1020,7 +1020,7 @@
         <v>0</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>0</v>
+        <v>1317.68</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>0</v>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="M69" s="4" t="inlineStr">
         <is>
-          <t>5 de 67</t>
+          <t>6 de 67</t>
         </is>
       </c>
       <c r="N69" s="4" t="inlineStr">
@@ -4849,7 +4849,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0</v>
+        <v>1317.68</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>1000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>17201.03</v>
+        <v>18518.71</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-13 10:30:15
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2508,7 +2508,7 @@
         <v>0</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>0</v>
+        <v>527.5</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0</v>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>0 de 67</t>
+          <t>1 de 67</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr">
@@ -5308,7 +5308,7 @@
         <v>3084.74</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>2118.8</v>
+        <v>2646.3</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>3000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>18518.71</v>
+        <v>19046.21</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-14 09:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -3894,7 +3894,7 @@
         <v>0</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>372.24</v>
+        <v>595.1900000000001</v>
       </c>
       <c r="L57" s="2" t="n">
         <v>0</v>
@@ -4017,7 +4017,7 @@
         <v>0</v>
       </c>
       <c r="L59" s="2" t="n">
-        <v>0</v>
+        <v>322.88</v>
       </c>
       <c r="M59" s="2" t="n">
         <v>0</v>
@@ -4626,7 +4626,7 @@
       </c>
       <c r="L69" s="4" t="inlineStr">
         <is>
-          <t>0 de 67</t>
+          <t>1 de 67</t>
         </is>
       </c>
       <c r="M69" s="4" t="inlineStr">
@@ -5821,7 +5821,7 @@
         <v>2814.28</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>372.24</v>
+        <v>595.1900000000001</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>4000</v>
@@ -5848,7 +5848,7 @@
         <v>2523.05</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0</v>
+        <v>322.88</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>2000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>19059.19</v>
+        <v>19605.02</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6051,7 +6051,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -6318,13 +6318,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>548.2</v>
+        <v>771.15</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>179.8</v>
+        <v>-43.14999999999998</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.7530219780219781</v>
+        <v>1.059271978021978</v>
       </c>
     </row>
     <row r="12">
@@ -6366,13 +6366,13 @@
         <v>2534</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0</v>
+        <v>322.88</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>2534</v>
+        <v>2211.12</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0</v>
+        <v>0.1274191002367798</v>
       </c>
     </row>
     <row r="14">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>19059.19</v>
+        <v>19605.02</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>62471.96000000001</v>
+        <v>61926.13</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2337657447490928</v>
+        <v>0.2404604865747632</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-14 14:30:16
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2220,7 +2220,7 @@
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>0</v>
+        <v>168.58</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
@@ -2916,7 +2916,7 @@
         <v>0</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0</v>
+        <v>259.28</v>
       </c>
       <c r="F41" s="2" t="n">
         <v>0</v>
@@ -2940,7 +2940,7 @@
         <v>0</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>-18.65</v>
+        <v>1613.08</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -4591,47 +4591,47 @@
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
+          <t>1 de 67</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
           <t>0 de 67</t>
         </is>
       </c>
-      <c r="F69" s="4" t="inlineStr">
+      <c r="G69" s="4" t="inlineStr">
         <is>
           <t>0 de 67</t>
         </is>
       </c>
-      <c r="G69" s="4" t="inlineStr">
+      <c r="H69" s="4" t="inlineStr">
         <is>
           <t>0 de 67</t>
         </is>
       </c>
-      <c r="H69" s="4" t="inlineStr">
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>1 de 67</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr">
         <is>
           <t>0 de 67</t>
         </is>
       </c>
-      <c r="I69" s="4" t="inlineStr">
+      <c r="K69" s="4" t="inlineStr">
+        <is>
+          <t>2 de 67</t>
+        </is>
+      </c>
+      <c r="L69" s="4" t="inlineStr">
         <is>
           <t>1 de 67</t>
         </is>
       </c>
-      <c r="J69" s="4" t="inlineStr">
-        <is>
-          <t>0 de 67</t>
-        </is>
-      </c>
-      <c r="K69" s="4" t="inlineStr">
-        <is>
-          <t>2 de 67</t>
-        </is>
-      </c>
-      <c r="L69" s="4" t="inlineStr">
-        <is>
-          <t>1 de 67</t>
-        </is>
-      </c>
       <c r="M69" s="4" t="inlineStr">
         <is>
-          <t>6 de 67</t>
+          <t>8 de 67</t>
         </is>
       </c>
       <c r="N69" s="4" t="inlineStr">
@@ -5227,7 +5227,7 @@
         <v>0</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0</v>
+        <v>168.58</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>3000</v>
@@ -5470,7 +5470,7 @@
         <v>13299.42</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>-5.67</v>
+        <v>1885.34</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>5000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>19605.02</v>
+        <v>21664.61</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6174,13 +6174,13 @@
         <v>199.5</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0</v>
+        <v>259.28</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>199.5</v>
+        <v>-59.77999999999997</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0</v>
+        <v>1.299649122807017</v>
       </c>
     </row>
     <row r="6">
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>6408.89</v>
+        <v>8209.200000000001</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>57201.26</v>
+        <v>55400.95</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.1007526314589731</v>
+        <v>0.1290548756762875</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>19605.02</v>
+        <v>21664.61</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>61926.13</v>
+        <v>59866.54</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2404604865747632</v>
+        <v>0.2657218744001526</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-14 16:30:16
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -1497,10 +1497,10 @@
         <v>0</v>
       </c>
       <c r="L17" s="2" t="n">
-        <v>0</v>
+        <v>571.54</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>72.03</v>
+        <v>137.59</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
@@ -1620,7 +1620,7 @@
         <v>0</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>147.07</v>
+        <v>472.16</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -4626,7 +4626,7 @@
       </c>
       <c r="L69" s="4" t="inlineStr">
         <is>
-          <t>1 de 67</t>
+          <t>2 de 67</t>
         </is>
       </c>
       <c r="M69" s="4" t="inlineStr">
@@ -5011,7 +5011,7 @@
         <v>2185.17</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>72.03</v>
+        <v>709.13</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>1500</v>
@@ -5065,7 +5065,7 @@
         <v>2184.08</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>147.07</v>
+        <v>472.16</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>2000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>21664.61</v>
+        <v>22626.8</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6366,13 +6366,13 @@
         <v>2534</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>322.88</v>
+        <v>894.42</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>2211.12</v>
+        <v>1639.58</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1274191002367798</v>
+        <v>0.3529676400947119</v>
       </c>
     </row>
     <row r="14">
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>8209.200000000001</v>
+        <v>8599.85</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>55400.95</v>
+        <v>55010.3</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.1290548756762875</v>
+        <v>0.1351961911738928</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>21664.61</v>
+        <v>22626.8</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>59866.54</v>
+        <v>58904.35000000001</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2657218744001526</v>
+        <v>0.2775233760348039</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-15 13:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -4554,7 +4554,7 @@
         <v>0</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>0</v>
+        <v>-7.44</v>
       </c>
       <c r="L68" s="2" t="n">
         <v>0</v>
@@ -5389,7 +5389,7 @@
         <v>7064.71</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>3008.2</v>
+        <v>2992.66</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>5000</v>
@@ -6010,7 +6010,7 @@
         <v>1286.02</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>34.48</v>
+        <v>27.04</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>1500</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>22626.8</v>
+        <v>22603.82</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6318,13 +6318,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>771.15</v>
+        <v>763.71</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-43.14999999999998</v>
+        <v>-35.71000000000004</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>1.059271978021978</v>
+        <v>1.049052197802198</v>
       </c>
     </row>
     <row r="12">
@@ -6342,13 +6342,13 @@
         <v>350</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>11259.23</v>
+        <v>11243.69</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-10909.23</v>
+        <v>-10893.69</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>32.16922857142857</v>
+        <v>32.12482857142857</v>
       </c>
     </row>
     <row r="13">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>22626.8</v>
+        <v>22603.82</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>58904.35000000001</v>
+        <v>58927.33</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2775233760348039</v>
+        <v>0.2772415205721985</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-15 16:30:16
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -5713,7 +5713,7 @@
         <v>-454.9</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>8251.030000000001</v>
+        <v>9338.66</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>2000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>22603.82</v>
+        <v>23691.45</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6342,13 +6342,13 @@
         <v>350</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>11243.69</v>
+        <v>12331.32</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-10893.69</v>
+        <v>-11981.32</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>32.12482857142857</v>
+        <v>35.23234285714285</v>
       </c>
     </row>
     <row r="13">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>22603.82</v>
+        <v>23691.45</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>58927.33</v>
+        <v>57839.7</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2772415205721985</v>
+        <v>0.2905815752629517</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-16 09:30:16
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2169,7 +2169,7 @@
         <v>0</v>
       </c>
       <c r="P28" s="2" t="n">
-        <v>0</v>
+        <v>25.85</v>
       </c>
       <c r="Q28" s="2" t="n">
         <v>0</v>
@@ -2940,7 +2940,7 @@
         <v>0</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>1613.08</v>
+        <v>4631.82</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -4646,7 +4646,7 @@
       </c>
       <c r="P69" s="4" t="inlineStr">
         <is>
-          <t>1 de 67</t>
+          <t>2 de 67</t>
         </is>
       </c>
       <c r="Q69" s="4" t="inlineStr">
@@ -5092,7 +5092,7 @@
         <v>4297.4</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>2738.84</v>
+        <v>2773.32</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>5000</v>
@@ -5200,7 +5200,7 @@
         <v>1728.65</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>34.48</v>
+        <v>60.33</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>3000</v>
@@ -5470,7 +5470,7 @@
         <v>13299.42</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>1885.34</v>
+        <v>4904.08</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>5000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>23691.45</v>
+        <v>26770.52</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6150,13 +6150,13 @@
         <v>5504</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>172.4</v>
+        <v>206.88</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>5331.6</v>
+        <v>5297.12</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.03132267441860465</v>
+        <v>0.03758720930232558</v>
       </c>
     </row>
     <row r="5">
@@ -6270,13 +6270,13 @@
         <v>250</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>12.98</v>
+        <v>38.83</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>237.02</v>
+        <v>211.17</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0.05192</v>
+        <v>0.15532</v>
       </c>
     </row>
     <row r="10">
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>8599.85</v>
+        <v>11618.59</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>55010.3</v>
+        <v>51991.56</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.1351961911738928</v>
+        <v>0.1826530828806409</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>23691.45</v>
+        <v>26770.52</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>57839.7</v>
+        <v>54760.63</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2905815752629517</v>
+        <v>0.3283471409393833</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-16 13:30:23
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -5821,7 +5821,7 @@
         <v>2814.28</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>595.1900000000001</v>
+        <v>1351.99</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>4000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>26770.52</v>
+        <v>27527.32</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6342,13 +6342,13 @@
         <v>350</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>12331.32</v>
+        <v>13088.12</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-11981.32</v>
+        <v>-12738.12</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>35.23234285714285</v>
+        <v>37.39462857142858</v>
       </c>
     </row>
     <row r="13">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>26770.52</v>
+        <v>27527.32</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>54760.63</v>
+        <v>54003.82999999999</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3283471409393833</v>
+        <v>0.3376294827191816</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-19 14:30:18
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2760,7 +2760,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>0</v>
+        <v>2012.49</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="M69" s="4" t="inlineStr">
         <is>
-          <t>8 de 67</t>
+          <t>9 de 67</t>
         </is>
       </c>
       <c r="N69" s="4" t="inlineStr">
@@ -5389,7 +5389,7 @@
         <v>7064.71</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>2992.66</v>
+        <v>5005.15</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>5000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>27527.32</v>
+        <v>29539.81</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>11618.59</v>
+        <v>13631.08</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>51991.56</v>
+        <v>49979.07</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.1826530828806409</v>
+        <v>0.2142909582826011</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>27527.32</v>
+        <v>29539.81</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>54003.82999999999</v>
+        <v>51991.34</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3376294827191816</v>
+        <v>0.3623131772334869</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-19 15:30:16
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -1620,7 +1620,7 @@
         <v>0</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>472.16</v>
+        <v>1029.47</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -5065,7 +5065,7 @@
         <v>2184.08</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>472.16</v>
+        <v>1302.71</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>2000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>29539.81</v>
+        <v>30370.36</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6150,13 +6150,13 @@
         <v>5504</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>206.88</v>
+        <v>480.12</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>5297.12</v>
+        <v>5023.88</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.03758720930232558</v>
+        <v>0.08723110465116279</v>
       </c>
     </row>
     <row r="5">
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>13631.08</v>
+        <v>14188.39</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>49979.07</v>
+        <v>49421.76</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.2142909582826011</v>
+        <v>0.2230522958993179</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>29539.81</v>
+        <v>30370.36</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>51991.34</v>
+        <v>51160.79</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3623131772334869</v>
+        <v>0.3725000812572863</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-20 09:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2757,10 +2757,10 @@
         <v>0</v>
       </c>
       <c r="L38" s="2" t="n">
-        <v>0</v>
+        <v>655.53</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>2012.49</v>
+        <v>3018.74</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -3825,10 +3825,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>0</v>
+        <v>513</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>0</v>
+        <v>142.95</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0</v>
@@ -3840,7 +3840,7 @@
         <v>0</v>
       </c>
       <c r="M56" s="2" t="n">
-        <v>0</v>
+        <v>2334.33</v>
       </c>
       <c r="N56" s="2" t="n">
         <v>0</v>
@@ -3849,7 +3849,7 @@
         <v>0</v>
       </c>
       <c r="P56" s="2" t="n">
-        <v>0</v>
+        <v>12.98</v>
       </c>
       <c r="Q56" s="2" t="n">
         <v>0</v>
@@ -4606,47 +4606,47 @@
       </c>
       <c r="H69" s="4" t="inlineStr">
         <is>
+          <t>1 de 67</t>
+        </is>
+      </c>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>2 de 67</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr">
+        <is>
           <t>0 de 67</t>
         </is>
       </c>
-      <c r="I69" s="4" t="inlineStr">
-        <is>
-          <t>1 de 67</t>
-        </is>
-      </c>
-      <c r="J69" s="4" t="inlineStr">
+      <c r="K69" s="4" t="inlineStr">
+        <is>
+          <t>2 de 67</t>
+        </is>
+      </c>
+      <c r="L69" s="4" t="inlineStr">
+        <is>
+          <t>3 de 67</t>
+        </is>
+      </c>
+      <c r="M69" s="4" t="inlineStr">
+        <is>
+          <t>10 de 67</t>
+        </is>
+      </c>
+      <c r="N69" s="4" t="inlineStr">
         <is>
           <t>0 de 67</t>
         </is>
       </c>
-      <c r="K69" s="4" t="inlineStr">
-        <is>
-          <t>2 de 67</t>
-        </is>
-      </c>
-      <c r="L69" s="4" t="inlineStr">
-        <is>
-          <t>2 de 67</t>
-        </is>
-      </c>
-      <c r="M69" s="4" t="inlineStr">
-        <is>
-          <t>9 de 67</t>
-        </is>
-      </c>
-      <c r="N69" s="4" t="inlineStr">
+      <c r="O69" s="4" t="inlineStr">
         <is>
           <t>0 de 67</t>
         </is>
       </c>
-      <c r="O69" s="4" t="inlineStr">
-        <is>
-          <t>0 de 67</t>
-        </is>
-      </c>
       <c r="P69" s="4" t="inlineStr">
         <is>
-          <t>2 de 67</t>
+          <t>3 de 67</t>
         </is>
       </c>
       <c r="Q69" s="4" t="inlineStr">
@@ -5389,7 +5389,7 @@
         <v>7064.71</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>5005.15</v>
+        <v>6666.93</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>5000</v>
@@ -5497,7 +5497,7 @@
         <v>0</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0</v>
+        <v>34.48</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>1500</v>
@@ -5794,7 +5794,7 @@
         <v>5232.14</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0</v>
+        <v>3003.26</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>3000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>30370.36</v>
+        <v>35069.88</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6150,13 +6150,13 @@
         <v>5504</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>480.12</v>
+        <v>514.6</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>5023.88</v>
+        <v>4989.4</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.08723110465116279</v>
+        <v>0.09349563953488373</v>
       </c>
     </row>
     <row r="5">
@@ -6222,13 +6222,13 @@
         <v>560</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0</v>
+        <v>513</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>560</v>
+        <v>47</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0</v>
+        <v>0.9160714285714285</v>
       </c>
     </row>
     <row r="8">
@@ -6246,13 +6246,13 @@
         <v>220</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>527.5</v>
+        <v>670.45</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-307.5</v>
+        <v>-450.45</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>2.397727272727273</v>
+        <v>3.0475</v>
       </c>
     </row>
     <row r="9">
@@ -6270,13 +6270,13 @@
         <v>250</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>38.83</v>
+        <v>51.81</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>211.17</v>
+        <v>198.19</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0.15532</v>
+        <v>0.20724</v>
       </c>
     </row>
     <row r="10">
@@ -6366,13 +6366,13 @@
         <v>2534</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>894.42</v>
+        <v>1549.95</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>1639.58</v>
+        <v>984.05</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.3529676400947119</v>
+        <v>0.6116614048934491</v>
       </c>
     </row>
     <row r="14">
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>14188.39</v>
+        <v>17528.97</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>49421.76</v>
+        <v>46081.18</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.2230522958993179</v>
+        <v>0.2755687575017509</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>30370.36</v>
+        <v>35069.88</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>51160.79</v>
+        <v>46461.27</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3725000812572863</v>
+        <v>0.4301408725376744</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-20 17:30:16
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2940,7 +2940,7 @@
         <v>0</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>4631.82</v>
+        <v>4554.42</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -3894,7 +3894,7 @@
         <v>0</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>595.1900000000001</v>
+        <v>557.4</v>
       </c>
       <c r="L57" s="2" t="n">
         <v>0</v>
@@ -5470,7 +5470,7 @@
         <v>13299.42</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>4904.08</v>
+        <v>4826.68</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>5000</v>
@@ -5713,7 +5713,7 @@
         <v>-454.9</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>9338.66</v>
+        <v>9320.82</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>2000</v>
@@ -5821,7 +5821,7 @@
         <v>2814.28</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>1351.99</v>
+        <v>1314.2</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>4000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>35069.88</v>
+        <v>34936.85</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6318,13 +6318,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>763.71</v>
+        <v>725.92</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-35.71000000000004</v>
+        <v>2.080000000000041</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>1.049052197802198</v>
+        <v>0.9971428571428571</v>
       </c>
     </row>
     <row r="12">
@@ -6342,13 +6342,13 @@
         <v>350</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>13088.12</v>
+        <v>13070.28</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-12738.12</v>
+        <v>-12720.28</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>37.39462857142858</v>
+        <v>37.34365714285715</v>
       </c>
     </row>
     <row r="13">
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>17528.97</v>
+        <v>17451.57</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>46081.18</v>
+        <v>46158.58</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.2755687575017509</v>
+        <v>0.2743519705581577</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>35069.88</v>
+        <v>34936.85</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>46461.27</v>
+        <v>46594.3</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.4301408725376744</v>
+        <v>0.4285092262282575</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-21 09:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -3840,7 +3840,7 @@
         <v>0</v>
       </c>
       <c r="M56" s="2" t="n">
-        <v>2334.33</v>
+        <v>4083.07</v>
       </c>
       <c r="N56" s="2" t="n">
         <v>0</v>
@@ -5794,7 +5794,7 @@
         <v>5232.14</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>3003.26</v>
+        <v>4752</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>3000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>34936.85</v>
+        <v>36685.59</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>17451.57</v>
+        <v>19200.31</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>46158.58</v>
+        <v>44409.84</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.2743519705581577</v>
+        <v>0.3018434951025898</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>34936.85</v>
+        <v>36685.59</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>46594.3</v>
+        <v>44845.56</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.4285092262282575</v>
+        <v>0.4499579608529991</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-21 17:30:16
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2820,7 +2820,7 @@
         <v>0</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>0</v>
+        <v>4502.81</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>0</v>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="M69" s="4" t="inlineStr">
         <is>
-          <t>11 de 67</t>
+          <t>12 de 67</t>
         </is>
       </c>
       <c r="N69" s="4" t="inlineStr">
@@ -5416,7 +5416,7 @@
         <v>10754.5</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0</v>
+        <v>4502.81</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>5000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>36710.43000000001</v>
+        <v>41213.24</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>19225.15</v>
+        <v>23727.96</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>44385</v>
+        <v>39882.19</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.3022339988193708</v>
+        <v>0.3730216011124011</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>36710.43</v>
+        <v>41213.24</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>44820.72</v>
+        <v>40317.91</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.4502626296820296</v>
+        <v>0.5054907234842143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-22 09:30:18
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2220,7 +2220,7 @@
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>168.58</v>
+        <v>211.58</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
@@ -5227,7 +5227,7 @@
         <v>0</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>168.58</v>
+        <v>211.58</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>3000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>41213.24</v>
+        <v>41256.24</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>23727.96</v>
+        <v>23770.96</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>39882.19</v>
+        <v>39839.19</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.3730216011124011</v>
+        <v>0.3736975938588417</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>41213.24</v>
+        <v>41256.24</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>40317.91</v>
+        <v>40274.91</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.5054907234842143</v>
+        <v>0.5060181292671574</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-22 10:30:16
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -5713,7 +5713,7 @@
         <v>-454.9</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>9320.82</v>
+        <v>9274.200000000001</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>2000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>41256.24</v>
+        <v>41209.62</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6342,13 +6342,13 @@
         <v>350</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>13070.28</v>
+        <v>13023.66</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-12720.28</v>
+        <v>-12673.66</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>37.34365714285715</v>
+        <v>37.21045714285714</v>
       </c>
     </row>
     <row r="13">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>41256.24</v>
+        <v>41209.62</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>40274.91</v>
+        <v>40321.53</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.5060181292671574</v>
+        <v>0.5054463232764409</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-22 16:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -1740,7 +1740,7 @@
         <v>0</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>2738.84</v>
+        <v>15330.78</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
@@ -4679,7 +4679,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -5092,7 +5092,7 @@
         <v>4297.4</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>2773.32</v>
+        <v>15365.26</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>5000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>41209.62</v>
+        <v>53801.56</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>23770.96</v>
+        <v>36362.9</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>39839.19</v>
+        <v>27247.25</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.3736975938588417</v>
+        <v>0.5716524799894357</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>41209.62</v>
+        <v>53801.56</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>40321.53</v>
+        <v>27729.59</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.5054463232764409</v>
+        <v>0.6598896250083557</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-23 09:30:19
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2940,7 +2940,7 @@
         <v>0</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>4554.42</v>
+        <v>6734.13</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -5470,7 +5470,7 @@
         <v>13299.42</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>4826.68</v>
+        <v>7006.39</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>5000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>53801.56</v>
+        <v>55981.27</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>36362.9</v>
+        <v>38542.61</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>27247.25</v>
+        <v>25067.54</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.5716524799894357</v>
+        <v>0.6059191811369726</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>53801.56</v>
+        <v>55981.27</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>27729.59</v>
+        <v>25549.88</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.6598896250083557</v>
+        <v>0.6866243147557713</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-26 08:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2940,7 +2940,7 @@
         <v>0</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>6734.13</v>
+        <v>6656.73</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -5470,7 +5470,7 @@
         <v>13299.42</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>7006.39</v>
+        <v>6928.99</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>5000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>55981.27</v>
+        <v>55903.87</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>38542.61</v>
+        <v>38465.21</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>25067.54</v>
+        <v>25144.94</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.6059191811369726</v>
+        <v>0.6047023941933795</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>55981.27</v>
+        <v>55903.87</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>25549.88</v>
+        <v>25627.28</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.6866243147557713</v>
+        <v>0.6856749843464737</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-27 11:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2940,7 +2940,7 @@
         <v>0</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>6656.73</v>
+        <v>6705.83</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -3594,7 +3594,7 @@
         <v>0</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>0</v>
+        <v>1003.32</v>
       </c>
       <c r="L52" s="2" t="n">
         <v>0</v>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="K69" s="4" t="inlineStr">
         <is>
-          <t>2 de 67</t>
+          <t>3 de 67</t>
         </is>
       </c>
       <c r="L69" s="4" t="inlineStr">
@@ -5470,7 +5470,7 @@
         <v>13299.42</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>6928.99</v>
+        <v>6978.09</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>5000</v>
@@ -5713,7 +5713,7 @@
         <v>-454.9</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>9274.200000000001</v>
+        <v>10277.52</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>2000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>55903.87</v>
+        <v>56956.29</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6318,13 +6318,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>725.92</v>
+        <v>1729.24</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2.080000000000041</v>
+        <v>-1001.24</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.9971428571428571</v>
+        <v>2.37532967032967</v>
       </c>
     </row>
     <row r="12">
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>38465.21</v>
+        <v>38514.31</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>25144.94</v>
+        <v>25095.84</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.6047023941933795</v>
+        <v>0.6054742835852454</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>55903.87</v>
+        <v>56956.28999999999</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>25627.28</v>
+        <v>24574.86</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.6856749843464737</v>
+        <v>0.6985831795577518</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-28 11:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -3594,7 +3594,7 @@
         <v>0</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>1003.32</v>
+        <v>966.17</v>
       </c>
       <c r="L52" s="2" t="n">
         <v>0</v>
@@ -5713,7 +5713,7 @@
         <v>-454.9</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>10277.52</v>
+        <v>10240.37</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>2000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>56956.29</v>
+        <v>56919.14</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6318,13 +6318,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1729.24</v>
+        <v>1692.09</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-1001.24</v>
+        <v>-964.0899999999999</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>2.37532967032967</v>
+        <v>2.324299450549451</v>
       </c>
     </row>
     <row r="12">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>56956.28999999999</v>
+        <v>56919.14</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>24574.86</v>
+        <v>24612.01</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.6985831795577518</v>
+        <v>0.6981275254917906</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-28 14:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -714,7 +714,7 @@
         <v>0</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>0</v>
+        <v>446.69</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>0</v>
@@ -2220,7 +2220,7 @@
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>211.58</v>
+        <v>1930.63</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="K69" s="4" t="inlineStr">
         <is>
-          <t>3 de 67</t>
+          <t>4 de 67</t>
         </is>
       </c>
       <c r="L69" s="4" t="inlineStr">
@@ -5227,7 +5227,7 @@
         <v>0</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>211.58</v>
+        <v>1930.63</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>3000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>56919.14</v>
+        <v>58638.19</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6318,13 +6318,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1692.09</v>
+        <v>2138.78</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-964.0899999999999</v>
+        <v>-1410.78</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>2.324299450549451</v>
+        <v>2.937884615384616</v>
       </c>
     </row>
     <row r="12">
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>38514.31</v>
+        <v>40233.36</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>25095.84</v>
+        <v>23376.79</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.6054742835852454</v>
+        <v>0.6324990587194025</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>56919.14</v>
+        <v>59084.88</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>24612.01</v>
+        <v>22446.27</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.6981275254917906</v>
+        <v>0.7246908696860036</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-28 16:30:16
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -1260,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0</v>
+        <v>1033.08</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="M69" s="4" t="inlineStr">
         <is>
-          <t>12 de 67</t>
+          <t>13 de 67</t>
         </is>
       </c>
       <c r="N69" s="4" t="inlineStr">
@@ -4930,7 +4930,7 @@
         <v>4420.8</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0</v>
+        <v>1033.08</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>2000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>61381.71</v>
+        <v>62414.79</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>42976.88</v>
+        <v>44009.96</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>20633.27</v>
+        <v>19600.19</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.6756292824336996</v>
+        <v>0.6918700867707434</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>61828.39999999999</v>
+        <v>62861.48</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>19702.75</v>
+        <v>18669.67</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.7583408304678642</v>
+        <v>0.7710118157293255</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-29 12:30:16
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -1620,7 +1620,7 @@
         <v>0</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>1029.47</v>
+        <v>2042.94</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -5065,7 +5065,7 @@
         <v>2184.08</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>1302.71</v>
+        <v>2316.18</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>2000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>62414.79</v>
+        <v>63428.26</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>44009.96</v>
+        <v>45023.43</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>19600.19</v>
+        <v>18586.72</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.6918700867707434</v>
+        <v>0.707802606973887</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>62861.48</v>
+        <v>63874.95</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>18669.67</v>
+        <v>17656.2</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.7710118157293255</v>
+        <v>0.7834422794232634</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-29 15:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2754,7 +2754,7 @@
         <v>0</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>0</v>
+        <v>2992.66</v>
       </c>
       <c r="L38" s="2" t="n">
         <v>655.53</v>
@@ -3594,7 +3594,7 @@
         <v>0</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>966.17</v>
+        <v>10240.37</v>
       </c>
       <c r="L52" s="2" t="n">
         <v>0</v>
@@ -3894,7 +3894,7 @@
         <v>0</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>557.4</v>
+        <v>1314.2</v>
       </c>
       <c r="L57" s="2" t="n">
         <v>0</v>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="K69" s="4" t="inlineStr">
         <is>
-          <t>4 de 67</t>
+          <t>5 de 67</t>
         </is>
       </c>
       <c r="L69" s="4" t="inlineStr">
@@ -6318,13 +6318,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>2138.78</v>
+        <v>15162.44</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-1410.78</v>
+        <v>-14434.44</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>2.937884615384616</v>
+        <v>20.82752747252747</v>
       </c>
     </row>
     <row r="12">
@@ -6342,13 +6342,13 @@
         <v>350</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>13023.66</v>
+        <v>0</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-12673.66</v>
+        <v>350</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>37.21045714285714</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Actualización automática 2026-10-30 09:30:17
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -2760,7 +2760,7 @@
         <v>655.53</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>3018.74</v>
+        <v>4494.93</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -5389,7 +5389,7 @@
         <v>7064.71</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>6666.93</v>
+        <v>8143.12</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>5000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>63428.26</v>
+        <v>64904.45</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>45023.43</v>
+        <v>46499.62</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>18586.72</v>
+        <v>17110.53</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.707802606973887</v>
+        <v>0.7310094379591936</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>63874.95</v>
+        <v>65351.14</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>17656.2</v>
+        <v>16180.01</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.7834422794232634</v>
+        <v>0.8015481199516995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-30 16:30:19
</commit_message>
<xml_diff>
--- a/data/CASTRO ALCIVAR EDA MARIA.xlsx
+++ b/data/CASTRO ALCIVAR EDA MARIA.xlsx
@@ -3225,7 +3225,7 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="I46" s="2" t="n">
         <v>0</v>
@@ -3540,7 +3540,7 @@
         <v>0</v>
       </c>
       <c r="M51" s="2" t="n">
-        <v>33.12</v>
+        <v>3119.19</v>
       </c>
       <c r="N51" s="2" t="n">
         <v>0</v>
@@ -3834,7 +3834,7 @@
         <v>0</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>0</v>
+        <v>17.91</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -4606,7 +4606,7 @@
       </c>
       <c r="H69" s="4" t="inlineStr">
         <is>
-          <t>1 de 67</t>
+          <t>2 de 67</t>
         </is>
       </c>
       <c r="I69" s="4" t="inlineStr">
@@ -4621,7 +4621,7 @@
       </c>
       <c r="K69" s="4" t="inlineStr">
         <is>
-          <t>5 de 67</t>
+          <t>6 de 67</t>
         </is>
       </c>
       <c r="L69" s="4" t="inlineStr">
@@ -5578,7 +5578,7 @@
         <v>1970.41</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>-47.38</v>
+        <v>42.62</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>1500</v>
@@ -5686,7 +5686,7 @@
         <v>4313.71</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>33.12</v>
+        <v>3119.19</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>5000</v>
@@ -5794,7 +5794,7 @@
         <v>5232.14</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>4752</v>
+        <v>4769.91</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>3000</v>
@@ -6027,7 +6027,7 @@
         <v>84322.79000000001</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>74560.55</v>
+        <v>77754.53</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>81531</v>
@@ -6222,13 +6222,13 @@
         <v>560</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>513</v>
+        <v>603</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>47</v>
+        <v>-43</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.9160714285714285</v>
+        <v>1.076785714285714</v>
       </c>
     </row>
     <row r="8">
@@ -6318,13 +6318,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>15180.35</v>
+        <v>15198.26</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-14452.35</v>
+        <v>-14470.26</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>20.85212912087912</v>
+        <v>20.87673076923077</v>
       </c>
     </row>
     <row r="12">
@@ -6390,13 +6390,13 @@
         <v>63610.15</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>55863.56</v>
+        <v>58949.63</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>7746.590000000004</v>
+        <v>4660.520000000004</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.8782177058221053</v>
+        <v>0.9267330764036871</v>
       </c>
     </row>
     <row r="15">
@@ -6433,13 +6433,13 @@
         <v>81531.14999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>75007.23999999999</v>
+        <v>78201.22</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>6523.910000000001</v>
+        <v>3329.930000000001</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.9199826078744135</v>
+        <v>0.95915757351638</v>
       </c>
     </row>
   </sheetData>

</xml_diff>